<commit_message>
Offerte 95mm²-Kabel (Excel) + gemeinsamer Offerten-Baukasten
- offerte_lib.py: extrahierter, konfigurierbarer Builder (Layout/Marke/
  Formeln identisch); unterstützt Miet- und Verkaufslayout, blendet die
  Faktor-Spalte aus, wenn nicht benötigt.
- build_template.py: nutzt jetzt offerte_lib (EKAG-Miete unverändert,
  reproduziert 16'609.27).
- build_offerte_kabel95.py + Offerte_Kabel_95mm.xlsx: neue Verkaufs-/
  Richtpreisofferte mit den 95mm²-Positionen aus Kabel_Mobil_in_Time_AG.pdf;
  GESAMT 11'146.50 (Steckendverschluss 12x, Kabel 3x, Regie 12x).
- offerte_to_pdf.py: liest Spaltenköpfe und Meta-Block dynamisch aus der
  Mappe -> passt das PDF automatisch an beide Offertentypen an.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014S9DaLfa6MkaKKTKAHq7pF
</commit_message>
<xml_diff>
--- a/offerten/Offerten_Master_Vorlage.xlsx
+++ b/offerten/Offerten_Master_Vorlage.xlsx
@@ -657,9 +657,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="6.5" customWidth="1" min="2" max="2"/>
+    <col width="7.5" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="7" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
@@ -808,7 +808,7 @@
     </row>
     <row r="14">
       <c r="A14" s="3">
-        <f>"Sehr geehrter "&amp;LEFT(A8,FIND(" ",A8)-1)&amp;" "&amp;MID(A8,FIND(" ",A8,FIND(" ",A8)+1)+1,99)</f>
+        <f>"Sehr geehrte"&amp;IF(LEFT(A8,4)="Frau"," Frau ",IF(LEFT(A8,4)="Herr","r Herr "," Damen und Herren"))&amp;IF(OR(LEFT(A8,4)="Frau",LEFT(A8,4)="Herr"),MID(A8,FIND(" ",A8&amp;" ",FIND(" ",A8&amp;" ")+1)+1,99),"")</f>
         <v/>
       </c>
     </row>
@@ -1496,7 +1496,7 @@
     <row r="45" ht="22" customHeight="1">
       <c r="A45" s="25" t="inlineStr">
         <is>
-          <t>Endbetrag (CHF)</t>
+          <t>Endbetrag</t>
         </is>
       </c>
       <c r="B45" s="26" t="n"/>
@@ -1854,7 +1854,7 @@
   <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="56" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
   </cols>
@@ -1872,7 +1872,7 @@
       </c>
       <c r="C1" s="35" t="inlineStr">
         <is>
-          <t>Einzelpreis/Woche (CHF)</t>
+          <t>Einzelpreis (CHF)</t>
         </is>
       </c>
     </row>

</xml_diff>